<commit_message>
Complete Phase 4 data quality
</commit_message>
<xml_diff>
--- a/04_Data_Quality/quality_summary.xlsx
+++ b/04_Data_Quality/quality_summary.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Issues" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trusted Validation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FK Validation" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -791,7 +792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -839,32 +840,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dim_customer</t>
+          <t>dim_account</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Leading/trailing whitespace in customer_name</t>
+          <t>Blank value in industry</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Trim whitespace</t>
+          <t>Convert blank to NULL before remediation</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>dim_employee</t>
+          <t>dim_customer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Leading/trailing whitespace in employee_name</t>
+          <t>Leading/trailing whitespace in customer_name</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -879,32 +880,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>dim_machine</t>
+          <t>dim_customer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Leading/trailing whitespace in machine_name</t>
+          <t>Blank value in country</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Trim whitespace</t>
+          <t>Convert blank to NULL before remediation</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>dim_product</t>
+          <t>dim_employee</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Leading/trailing whitespace in product_name</t>
+          <t>Leading/trailing whitespace in employee_name</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -919,61 +920,61 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dim_supplier</t>
+          <t>dim_location</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Leading/trailing whitespace in supplier_name</t>
+          <t>Blank value in city</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Trim whitespace</t>
+          <t>Convert blank to NULL before remediation</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dim_customer</t>
+          <t>dim_machine</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Missing country</t>
+          <t>Leading/trailing whitespace in machine_name</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fill with Unknown</t>
+          <t>Trim whitespace</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dim_customer</t>
+          <t>dim_product</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Invalid customer segment</t>
+          <t>Leading/trailing whitespace in product_name</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Replace with Unknown</t>
+          <t>Trim whitespace</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -984,12 +985,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Missing subcategory</t>
+          <t>Blank value in subcategory</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fill with Unknown</t>
+          <t>Convert blank to NULL before remediation</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1004,16 +1005,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Missing supplier category</t>
+          <t>Leading/trailing whitespace in supplier_name</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fill with Unknown</t>
+          <t>Trim whitespace</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -1024,52 +1025,52 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Invalid supplier category</t>
+          <t>Blank value in supplier_category</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Replace with Unknown</t>
+          <t>Convert blank to NULL before remediation</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dim_location</t>
+          <t>fact_budget</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Invalid location type</t>
+          <t>Blank value in budget_category</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Replace with Unknown</t>
+          <t>Convert blank to NULL before remediation</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dim_machine</t>
+          <t>fact_emissions</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Invalid machine status</t>
+          <t>Blank value in emissions_category</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Replace with Unknown</t>
+          <t>Convert blank to NULL before remediation</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1084,12 +1085,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Missing maintenance type</t>
+          <t>Blank value in maintenance_type</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fill with Unknown</t>
+          <t>Convert blank to NULL before remediation</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1099,141 +1100,141 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fact_sales</t>
+          <t>dim_account</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Duplicate transaction IDs</t>
+          <t>Missing required text value in industry</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Remove duplicate rows</t>
+          <t>Fill with Unknown</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>500</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>fact_production</t>
+          <t>dim_customer</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Duplicate production IDs</t>
+          <t>Missing required text value in country</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Remove duplicate rows</t>
+          <t>Fill with Unknown</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>fact_financial_transaction</t>
+          <t>dim_supplier</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Duplicate transaction IDs</t>
+          <t>Missing required text value in supplier_category</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Remove duplicate rows</t>
+          <t>Fill with Unknown</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>300</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>fact_sales</t>
+          <t>dim_location</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Invalid customer reference</t>
+          <t>Missing required text value in city</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Remove row</t>
+          <t>Fill with Unknown</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>500</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>fact_inventory</t>
+          <t>fact_maintenance</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Invalid product reference</t>
+          <t>Missing required text value in maintenance_type</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Remove row</t>
+          <t>Fill with Unknown</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>fact_energy</t>
+          <t>fact_budget</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Invalid machine reference</t>
+          <t>Missing required text value in budget_category</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Remove row</t>
+          <t>Fill with Unknown</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>fact_maintenance</t>
+          <t>fact_emissions</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Invalid employee reference</t>
+          <t>Missing required text value in emissions_category</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Remove row</t>
+          <t>Fill with Unknown</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23">
@@ -1244,152 +1245,152 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Negative sales quantity</t>
+          <t>Duplicate primary key in sales_key</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Remove row</t>
+          <t>Remove duplicate row</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>fact_inventory</t>
+          <t>fact_production</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Negative issued quantity</t>
+          <t>Duplicate primary key in production_key</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Remove row</t>
+          <t>Remove duplicate row</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>fact_energy</t>
+          <t>fact_financial_transaction</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Negative energy consumption</t>
+          <t>Duplicate primary key in financial_transaction_key</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Remove row</t>
+          <t>Remove duplicate row</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>fact_waste</t>
+          <t>dim_customer</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Negative waste quantity</t>
+          <t>Invalid customer segment</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Remove row</t>
+          <t>Replace with Unknown</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>fact_sales</t>
+          <t>dim_supplier</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Revenue reconciliation failure</t>
+          <t>Invalid supplier category</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Recalculate revenue</t>
+          <t>Replace with Unknown</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>499</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>fact_inventory</t>
+          <t>dim_location</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Closing quantity reconciliation failure</t>
+          <t>Invalid location type</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Recalculate closing quantity</t>
+          <t>Replace with Unknown</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>500</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>fact_production</t>
+          <t>fact_sales</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Defect quantity greater than produced quantity</t>
+          <t>Negative value in quantity</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Cap defects at produced quantity</t>
+          <t>Remove row</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>198</v>
+        <v>499</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>fact_production</t>
+          <t>fact_energy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Production outlier</t>
+          <t>Negative value in energy_consumption</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Retain for investigation</t>
+          <t>Remove row</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1399,20 +1400,220 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>fact_waste</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Negative value in waste_quantity</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Remove row</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>fact_inventory</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Negative value in issued_quantity</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Remove row</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>fact_sales</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Invalid foreign key: customer_key -&gt; dim_customer.customer_key</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Remove row</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>fact_maintenance</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Invalid foreign key: employee_key -&gt; dim_employee.employee_key</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Remove row</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>fact_energy</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Invalid foreign key: machine_key -&gt; dim_machine.machine_key</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Remove row</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>fact_inventory</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Invalid foreign key: product_key -&gt; dim_product.product_key</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Remove row</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>fact_sales</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Revenue reconciliation failure</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Recalculate revenue</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>fact_inventory</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Closing quantity reconciliation failure</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Recalculate closing quantity</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>fact_production</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Defect quantity greater than produced quantity</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Cap defects at produced quantity</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>fact_production</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Production outlier</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Retain for investigation</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>fact_financial_transaction</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>Financial transaction outlier</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Retain for investigation</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D41" t="n">
         <v>118</v>
       </c>
     </row>
@@ -1427,7 +1628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1438,12 +1639,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Null Values</t>
+          <t>Rows</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Total Nulls</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Nulls</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unexpected Nulls</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Duplicate Rows</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -1454,10 +1675,24 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>1000</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1467,10 +1702,24 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1480,10 +1729,24 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>2557</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1493,10 +1756,24 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1506,10 +1783,24 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1519,10 +1810,24 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1532,10 +1837,24 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1545,10 +1864,24 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1558,10 +1891,24 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>20</v>
+        <v>20000</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1571,10 +1918,24 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20</v>
+        <v>100000</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1584,10 +1945,24 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>99800</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1597,10 +1972,24 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1610,10 +1999,24 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>499000</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1623,10 +2026,24 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>49950</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1636,10 +2053,24 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1649,10 +2080,24 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>499002</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1662,10 +2107,1060 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>99900</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Child Dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Child Column</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Parent Dataset</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Parent Column</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Invalid References</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dim_customer</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>account_key</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>dim_account</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>account_key</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dim_product</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>supplier_key</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>dim_supplier</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>supplier_key</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dim_employee</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dim_machine</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>fact_sales</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dim_date</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fact_sales</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>customer_key</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dim_customer</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>customer_key</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fact_sales</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>product_key</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>dim_product</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>product_key</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>fact_sales</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>fact_production</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>dim_date</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>fact_production</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>product_key</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>dim_product</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>product_key</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>fact_production</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>fact_production</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>machine_key</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>dim_machine</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>machine_key</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>fact_production</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>employee_key</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>dim_employee</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>employee_key</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>fact_maintenance</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>dim_date</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>fact_maintenance</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>fact_maintenance</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>machine_key</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>dim_machine</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>machine_key</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>fact_maintenance</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>employee_key</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>dim_employee</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>employee_key</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>fact_financial_transaction</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>dim_date</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>fact_financial_transaction</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>account_key</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>dim_account</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>account_key</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>fact_financial_transaction</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>fact_budget</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>dim_date</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>fact_budget</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>account_key</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>dim_account</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>account_key</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>fact_budget</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>fact_energy</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>dim_date</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>fact_energy</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>fact_energy</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>machine_key</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>dim_machine</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>machine_key</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>fact_emissions</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>dim_date</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>fact_emissions</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>fact_waste</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>dim_date</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fact_waste</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>fact_inventory</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>dim_date</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>date_key</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>fact_inventory</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>product_key</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>dim_product</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>product_key</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>fact_inventory</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>dim_location</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>location_key</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>